<commit_message>
Update TVAR model outputs (2026-09-01)
</commit_message>
<xml_diff>
--- a/tvar/DataCompleteLatest.xlsx
+++ b/tvar/DataCompleteLatest.xlsx
@@ -37,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="60" uniqueCount="37">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" count="69" uniqueCount="37">
   <si>
     <t>Pi</t>
   </si>
@@ -9508,7 +9508,7 @@
         <v>46113</v>
       </c>
       <c r="B319" s="0">
-        <v>5.1311267636182265</v>
+        <v>5.2529055154485462</v>
       </c>
       <c r="C319" s="0">
         <v>2.2172000000000001</v>
@@ -9533,7 +9533,9 @@
         <v>46204</v>
       </c>
       <c r="B320" s="0"/>
-      <c r="C320" s="0"/>
+      <c r="C320" s="0">
+        <v>2.2000000000000002</v>
+      </c>
       <c r="D320" s="0">
         <v>3.73</v>
       </c>

</xml_diff>